<commit_message>
Salinity Model tunning parameters
</commit_message>
<xml_diff>
--- a/4-tables-and-figures/data_summary.xlsx
+++ b/4-tables-and-figures/data_summary.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\courses\capstone4ds_Fazio\4-tables-and-figures\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F1BA009B-9DEA-4D68-A753-5AA75E835509}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{15814006-B693-4D03-A3BD-6BAFB097A83E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="17385" xr2:uid="{5551CE1F-312C-4372-A693-7C40E2554840}"/>
+    <workbookView xWindow="1215" yWindow="2385" windowWidth="21600" windowHeight="12645" xr2:uid="{5551CE1F-312C-4372-A693-7C40E2554840}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -59,12 +59,6 @@
     <t>Depth / bathymetry</t>
   </si>
   <si>
-    <t>Count</t>
-  </si>
-  <si>
-    <t>Resolution</t>
-  </si>
-  <si>
     <t>Source</t>
   </si>
   <si>
@@ -83,19 +77,25 @@
     <t>Chlorophyll a</t>
   </si>
   <si>
-    <t>@wqp_2026</t>
-  </si>
-  <si>
     <t>Oyster Reefs</t>
   </si>
   <si>
     <t>Polygon</t>
   </si>
   <si>
-    <t>@FWC2026Oysters</t>
-  </si>
-  <si>
-    <t>@PPBEP_OysterRestoration</t>
+    <t>Processed Count</t>
+  </si>
+  <si>
+    <t># of Records</t>
+  </si>
+  <si>
+    <t>[@wqp_2026]</t>
+  </si>
+  <si>
+    <t>[@FWC2026Oysters]</t>
+  </si>
+  <si>
+    <t>[@PPBEP_OysterRestoration]</t>
   </si>
 </sst>
 </file>
@@ -490,8 +490,7 @@
   <cols>
     <col min="1" max="1" width="29.28515625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="13.85546875" customWidth="1"/>
-    <col min="3" max="3" width="17.140625" customWidth="1"/>
-    <col min="4" max="4" width="19.42578125" customWidth="1"/>
+    <col min="3" max="4" width="17.140625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -502,13 +501,13 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
+        <v>15</v>
+      </c>
+      <c r="D1" t="s">
+        <v>14</v>
+      </c>
+      <c r="E1" t="s">
         <v>6</v>
-      </c>
-      <c r="D1" t="s">
-        <v>7</v>
-      </c>
-      <c r="E1" t="s">
-        <v>8</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
@@ -516,21 +515,33 @@
         <v>2</v>
       </c>
       <c r="B2" t="s">
-        <v>9</v>
+        <v>7</v>
+      </c>
+      <c r="C2">
+        <v>6992</v>
+      </c>
+      <c r="D2">
+        <v>95</v>
       </c>
       <c r="E2" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B3" t="s">
-        <v>9</v>
+        <v>7</v>
+      </c>
+      <c r="C3">
+        <v>7159</v>
+      </c>
+      <c r="D3">
+        <v>100</v>
       </c>
       <c r="E3" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
@@ -538,7 +549,7 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="E4" s="2" t="s">
         <v>18</v>
@@ -549,10 +560,16 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>9</v>
+        <v>7</v>
+      </c>
+      <c r="C5">
+        <v>6261</v>
+      </c>
+      <c r="D5">
+        <v>99</v>
       </c>
       <c r="E5" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
@@ -560,40 +577,58 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="E6" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B7" t="s">
-        <v>9</v>
+        <v>7</v>
+      </c>
+      <c r="C7">
+        <v>3402</v>
+      </c>
+      <c r="D7">
+        <v>75</v>
       </c>
       <c r="E7" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B8" t="s">
-        <v>9</v>
+        <v>7</v>
+      </c>
+      <c r="C8">
+        <v>1847</v>
+      </c>
+      <c r="D8">
+        <v>44</v>
       </c>
       <c r="E8" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="B9" t="s">
-        <v>16</v>
+        <v>13</v>
+      </c>
+      <c r="C9">
+        <v>443</v>
+      </c>
+      <c r="D9">
+        <v>443</v>
       </c>
       <c r="E9" s="1" t="s">
         <v>17</v>

</xml_diff>